<commit_message>
Add http request to esp32 and build the esp32 server
</commit_message>
<xml_diff>
--- a/database/users.xlsx
+++ b/database/users.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -477,6 +477,38 @@
       <c r="F2" t="inlineStr">
         <is>
           <t>2026-07-09 14:18:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Try Boukheang</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>2024476</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Cyber Security</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Student</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>images/20260713_143607.jpg</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2026-07-13 14:36:20</t>
         </is>
       </c>
     </row>

</xml_diff>